<commit_message>
Hotel Checklists Kit Pro (EN): revisión final adversarial — 1 B, 3 M, 15 m; remontado, gates VERDE 8/0
B1 spa: el cierre ya no apaga la filtración ni la desinfección del hot tub (MAHC 2024 §5.12.1.1).
M1 simulacro trimestral en cada turno (IFC Table 405.2, R-1); M2 hot tub, no piscina, a 95-100 °F;
M3 sneeze guard, plato limpio y buffet vigilado (FDA 3-306.11, 3-304.16, 3-306.13).
Menores: títulos y orden de uso del 18/19, nº de informe, carnés, calendario, host stand.
Idempotencia 0, autotest 19/19, censo 0 defectos. Erratas del ES en hotel/ERRATAS-ES.md.

Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/hotel-checklist-templates/01-hotel-breakfast-buffet-checklists.xlsx
+++ b/astro-site/public/dl/hotel-checklist-templates/01-hotel-breakfast-buffet-checklists.xlsx
@@ -1321,7 +1321,7 @@
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>Set up the hot station: chafing dishes, pans, serving spoons</t>
+          <t>Set up the hot station: chafing dishes, pans and serving spoons, behind the sneeze guard (FDA 3-306.11)</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>Keep the buffet clean at all times: wipe up spills immediately</t>
+          <t>Keep the buffet watched by trained staff and clean at all times (FDA 3-306.13): wipe up spills immediately</t>
         </is>
       </c>
       <c r="C48" s="16" t="inlineStr">

</xml_diff>